<commit_message>
Added Additional Week 2 Exercises
</commit_message>
<xml_diff>
--- a/week-02/In Class Practice Files/Normalization Practice Exercise 1.xlsx
+++ b/week-02/In Class Practice Files/Normalization Practice Exercise 1.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swaid\Documents\DataAnalytics\week-02\In Class Practice Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6667A106-31AF-46FD-A798-ED006E4CE71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D721AE87-0024-46E9-AC96-DD091151D7D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7EACDFCF-20A2-4EFD-B44F-0CEF36CC6117}"/>
+    <workbookView xWindow="360" yWindow="3315" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{7EACDFCF-20A2-4EFD-B44F-0CEF36CC6117}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="UNF" sheetId="4" r:id="rId1"/>
+    <sheet name="1NF" sheetId="2" r:id="rId2"/>
+    <sheet name="2NF" sheetId="3" r:id="rId3"/>
+    <sheet name="3NF" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,10 +41,89 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="22">
+  <si>
+    <t>StudentID</t>
+  </si>
+  <si>
+    <t>Course</t>
+  </si>
+  <si>
+    <t>StudentName</t>
+  </si>
+  <si>
+    <t>Instructor</t>
+  </si>
+  <si>
+    <t>InstructorPhone</t>
+  </si>
+  <si>
+    <t>Alice Johnson</t>
+  </si>
+  <si>
+    <t>Dr. Smith</t>
+  </si>
+  <si>
+    <t>555-1111</t>
+  </si>
+  <si>
+    <t>Bob Lee</t>
+  </si>
+  <si>
+    <t>Excel</t>
+  </si>
+  <si>
+    <t>Dr. Brown</t>
+  </si>
+  <si>
+    <t>555-2222</t>
+  </si>
+  <si>
+    <t>Maria Gomez</t>
+  </si>
+  <si>
+    <t>James Kim</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>Dr. White</t>
+  </si>
+  <si>
+    <t>555-3333</t>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
+  <si>
+    <t>CourseInfo</t>
+  </si>
+  <si>
+    <t>SQL, Python</t>
+  </si>
+  <si>
+    <t>SQL, Excel, Python</t>
+  </si>
+  <si>
+    <t>Instructor Phone</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -57,7 +139,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,12 +147,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,10 +510,586 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1B5343-AD34-4EA7-ACB1-6F89D67695F4}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E17A779-1B02-4D53-AD3E-3DDD5AC6661A}">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>101</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>102</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>103</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>104</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C191AF3-AFCB-4950-BB31-2990A5EA5994}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>101</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>101</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>102</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>103</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>103</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>104</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82766ADC-A5EB-4B09-A937-6A7EAA9D4B73}">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>101</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="3">
+        <v>101</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>102</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3">
+        <v>101</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>103</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3">
+        <v>102</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>104</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="3">
+        <v>103</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E6" s="3">
+        <v>103</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E7" s="3">
+        <v>103</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E8" s="3">
+        <v>104</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82F74EEF-DA51-4596-9AFD-7E4B241AE1AF}">
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" s="1"/>
+      <c r="M1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>101</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="3">
+        <v>101</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>102</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M3" s="3">
+        <v>101</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>103</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="3">
+        <v>102</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>104</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" s="3">
+        <v>103</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M6" s="3">
+        <v>103</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M7" s="3">
+        <v>103</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M8" s="3">
+        <v>104</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>